<commit_message>
Mark Phase 2 items OE-02, OE-03 as resolved in audit workbook
Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Content_Integrity_Pipeline_Audit.xlsx
+++ b/Content_Integrity_Pipeline_Audit.xlsx
@@ -1775,69 +1775,69 @@
       </c>
     </row>
     <row r="2" ht="39.75" customHeight="1" s="22">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="23" t="inlineStr">
         <is>
           <t>Pipeline / Subsystem</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="23" t="inlineStr">
         <is>
           <t>Data Flow (Input → Output)</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="23" t="inlineStr">
         <is>
           <t>Entry Point</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="23" t="inlineStr">
         <is>
           <t>Exit Point</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="23" t="inlineStr">
         <is>
           <t>Primary Tech Stack</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="23" t="inlineStr">
         <is>
           <t># Components
 Audited</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="23" t="inlineStr">
         <is>
           <t># Keep</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="I2" s="23" t="inlineStr">
         <is>
           <t># Enhance</t>
         </is>
       </c>
-      <c r="J2" s="3" t="inlineStr">
+      <c r="J2" s="23" t="inlineStr">
         <is>
           <t># Remove</t>
         </is>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" s="23" t="inlineStr">
         <is>
           <t>Health Index %</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="L2" s="23" t="inlineStr">
         <is>
           <t>High/Critical
 Issues Open</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="M2" s="23" t="inlineStr">
         <is>
           <t>Current Architectural Bottleneck</t>
         </is>
@@ -1854,22 +1854,22 @@
           <t>XML Ingestion &amp; Record Parsing</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="24" t="inlineStr">
         <is>
           <t>Raw submission XML → ParsedRecord objects (id, title, abstract, sections, authors, affiliations, trial IDs)</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="24" t="inlineStr">
         <is>
           <t>Batch of ~6,000 ASCO XML abstracts</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="24" t="inlineStr">
         <is>
           <t>ParsedRecord list consumed by every detector</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F3" s="24" t="inlineStr">
         <is>
           <t>lxml; Python re</t>
         </is>
@@ -1898,7 +1898,7 @@
         <f>COUNTIFS('Overengineering Log'!$B:$B,"*"&amp;$B3&amp;"*",'Overengineering Log'!$F:$F,"Critical")+COUNTIFS('Overengineering Log'!$B:$B,"*"&amp;$B3&amp;"*",'Overengineering Log'!$F:$F,"High")</f>
         <v/>
       </c>
-      <c r="M3" s="9" t="inlineStr">
+      <c r="M3" s="24" t="inlineStr">
         <is>
           <t>Undocumented/duplicated pre-processing (dedup, sentence-splitting) creates invisible correctness risk shared by every downstream detector.</t>
         </is>
@@ -1976,22 +1976,22 @@
           <t>Template Detection (Cross-Author)</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="24" t="inlineStr">
         <is>
           <t>ParsedRecord[] → original/normalized/masked text → candidate pairs → pair classification → Templating flag + Template Evidence rows</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="24" t="inlineStr">
         <is>
           <t>Title, abstract, sections per record</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="24" t="inlineStr">
         <is>
           <t>Templating (Cross-Author) flag + Template Evidence sheet rows</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="F5" s="24" t="inlineStr">
         <is>
           <t>Python regex; difflib.SequenceMatcher; BLAKE2b/SHA-256 fingerprints; optional HF Transformers (PubMedBERT) / SciSpaCy</t>
         </is>
@@ -2020,7 +2020,7 @@
         <f>COUNTIFS('Overengineering Log'!$B:$B,"*"&amp;$B5&amp;"*",'Overengineering Log'!$F:$F,"Critical")+COUNTIFS('Overengineering Log'!$B:$B,"*"&amp;$B5&amp;"*",'Overengineering Log'!$F:$F,"High")</f>
         <v/>
       </c>
-      <c r="M5" s="9" t="inlineStr">
+      <c r="M5" s="24" t="inlineStr">
         <is>
           <t>Pairwise candidate comparison scales only to a single annual batch; a fully-built family-clustering capability sits unused.</t>
         </is>
@@ -2098,22 +2098,22 @@
           <t>Tortured Phrase Detection</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="24" t="inlineStr">
         <is>
           <t>Title/abstract → dictionary+regex candidates (known) &amp; sentence-level GPT-OSS candidates (new) → validated findings</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="24" t="inlineStr">
         <is>
           <t>Title, abstract text</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="24" t="inlineStr">
         <is>
           <t>Confirmed tortured-phrase findings; new-phrase discovery candidates</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F7" s="24" t="inlineStr">
         <is>
           <t>Python re; CSV rule dictionary; GPT-OSS 20B (temperature=0)</t>
         </is>
@@ -2142,7 +2142,7 @@
         <f>COUNTIFS('Overengineering Log'!$B:$B,"*"&amp;$B7&amp;"*",'Overengineering Log'!$F:$F,"Critical")+COUNTIFS('Overengineering Log'!$B:$B,"*"&amp;$B7&amp;"*",'Overengineering Log'!$F:$F,"High")</f>
         <v/>
       </c>
-      <c r="M7" s="9" t="inlineStr">
+      <c r="M7" s="24" t="inlineStr">
         <is>
           <t>Correctness bug: the proximity operator (~N) in dictionary syntax is parsed but never enforced.</t>
         </is>
@@ -2220,22 +2220,22 @@
           <t>Design Contradiction</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="24" t="inlineStr">
         <is>
           <t>Title + abstract sections → regex design-attribute claims → fixed incompatibility rules → component/context suppression → optional LLM annotation</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="24" t="inlineStr">
         <is>
           <t>Title, abstract sections</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="24" t="inlineStr">
         <is>
           <t>Design contradiction findings (+ optional non-gating LLM annotation)</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="F9" s="24" t="inlineStr">
         <is>
           <t>Python re; itertools; optional GPT-OSS 20B via IntelliHub</t>
         </is>
@@ -2264,7 +2264,7 @@
         <f>COUNTIFS('Overengineering Log'!$B:$B,"*"&amp;$B9&amp;"*",'Overengineering Log'!$F:$F,"Critical")+COUNTIFS('Overengineering Log'!$B:$B,"*"&amp;$B9&amp;"*",'Overengineering Log'!$F:$F,"High")</f>
         <v/>
       </c>
-      <c r="M9" s="9" t="inlineStr">
+      <c r="M9" s="24" t="inlineStr">
         <is>
           <t>LLM validation result is computed but never gates the surfaced flag — inconsistent with the other two LLM-validated checks.</t>
         </is>
@@ -2342,22 +2342,22 @@
           <t>Consolidated Workbook / Reporting</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="24" t="inlineStr">
         <is>
           <t>Finding[] across all six checks → All Abstracts / Check Detail / Template Evidence sheets in one XLSX</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="24" t="inlineStr">
         <is>
           <t>Findings from P3–P8</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E11" s="24" t="inlineStr">
         <is>
           <t>Editor-facing consolidated .xlsx workbook</t>
         </is>
       </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="F11" s="24" t="inlineStr">
         <is>
           <t>XLSX export layer per PRD (openpyxl/pandas-style)</t>
         </is>
@@ -2386,7 +2386,7 @@
         <f>COUNTIFS('Overengineering Log'!$B:$B,"*"&amp;$B11&amp;"*",'Overengineering Log'!$F:$F,"Critical")+COUNTIFS('Overengineering Log'!$B:$B,"*"&amp;$B11&amp;"*",'Overengineering Log'!$F:$F,"High")</f>
         <v/>
       </c>
-      <c r="M11" s="9" t="inlineStr">
+      <c r="M11" s="24" t="inlineStr">
         <is>
           <t>Multiple structured fields computed internally (numeric deltas, trial metadata, validation reasons) are silently dropped before export.</t>
         </is>
@@ -3485,42 +3485,42 @@
       </c>
     </row>
     <row r="2" ht="24" customHeight="1" s="22">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>Pipeline Name</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="23" t="inlineStr">
         <is>
           <t>Component / Module</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="23" t="inlineStr">
         <is>
           <t>Current Implementation</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="23" t="inlineStr">
         <is>
           <t>Real-World Viability</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="23" t="inlineStr">
         <is>
           <t>Verdict</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="23" t="inlineStr">
         <is>
           <t>Action Items</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="23" t="inlineStr">
         <is>
           <t>Source Reference</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="23" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
@@ -3537,12 +3537,12 @@
           <t>XML Ingestion &amp; Record Parsing</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>XML Parser (lxml)</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="C3" s="24" t="inlineStr">
         <is>
           <t>lxml parses raw submission XML into ParsedRecord objects; extracts ID, title, abstract, structured sections, authors, affiliations, trial IDs.</t>
         </is>
@@ -3557,12 +3557,12 @@
           <t>Enhance</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="F3" s="24" t="inlineStr">
         <is>
           <t>Add a schema-tolerant fallback (recover=True or a secondary parser) plus structured parse-failure logging with reason codes, instead of the current 'remove records whose parsing failed' silent drop.</t>
         </is>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="G3" s="24" t="inlineStr">
         <is>
           <t>Template Detection §2; Numerical/Design/Trial §1</t>
         </is>
@@ -3621,12 +3621,12 @@
           <t>XML Ingestion &amp; Record Parsing</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Sentence Splitter (regex `(?&lt;=[.!?])\s+`)</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="24" t="inlineStr">
         <is>
           <t>Naive punctuation-lookbehind regex, independently reimplemented in Numerical, Design, and Clinical Trial detectors (and implied elsewhere).</t>
         </is>
@@ -3641,12 +3641,12 @@
           <t>Enhance</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="F5" s="24" t="inlineStr">
         <is>
           <t>Extract one shared, abbreviation-aware sentence tokenizer (e.g. pySBD or a spaCy rule-based sentencizer) and delete the per-pipeline copies.</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="G5" s="24" t="inlineStr">
         <is>
           <t>Numerical/Design/Trial §1 (shared pipeline behaviour)</t>
         </is>
@@ -3710,12 +3710,12 @@
           <t>XML Ingestion &amp; Record Parsing</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>Failed/Empty Record Filtering</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="24" t="inlineStr">
         <is>
           <t>Records with failed parsing or no usable title/abstract text are removed before detectors run.</t>
         </is>
@@ -3730,12 +3730,12 @@
           <t>Keep</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
+      <c r="F7" s="24" t="inlineStr">
         <is>
           <t>Emit exclusion counts + reasons into run metadata instead of a silent drop -- the PRD explicitly requires the workbook to 'show all abstracts and run metadata' even when nothing is found.</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="G7" s="24" t="inlineStr">
         <is>
           <t>Numerical/Design/Trial §1; PRD v1 §12 edge cases</t>
         </is>
@@ -3799,12 +3799,12 @@
           <t>Orchestration &amp; Risk Aggregation</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="24" t="inlineStr">
         <is>
           <t>Cross-Pipeline Threshold / Config Management</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="24" t="inlineStr">
         <is>
           <t>At least 15 numeric thresholds (similarity cutoffs, word-count minimums, confidence mappings, timeouts, tolerances) are hardcoded independently inside each detector module.</t>
         </is>
@@ -3819,12 +3819,12 @@
           <t>Keep</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="F9" s="24" t="inlineStr">
         <is>
           <t>Centralize into one versioned config, extending the dictionary/pattern-version discipline already used for tortured phrases to every threshold.</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="G9" s="24" t="inlineStr">
         <is>
           <t>Cross-pipeline (Template §4, Tortured Phrase §13, Numerical §5, Trial §21)</t>
         </is>
@@ -3893,12 +3893,12 @@
           <t>Orchestration &amp; Risk Aggregation</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Run Metadata &amp; Dictionary Versioning</t>
         </is>
       </c>
-      <c r="C11" s="9" t="inlineStr">
+      <c r="C11" s="24" t="inlineStr">
         <is>
           <t>PRD risk mitigation calls for storing dictionary version and screening-run metadata; only documented in detail for the tortured-phrase CSV.</t>
         </is>
@@ -3913,12 +3913,12 @@
           <t>Keep</t>
         </is>
       </c>
-      <c r="F11" s="9" t="inlineStr">
+      <c r="F11" s="24" t="inlineStr">
         <is>
           <t>Confirm and extend version stamping to the LLM-trace YAML catalogue and the design-contradiction rule table so every rule source is auditable the same way.</t>
         </is>
       </c>
-      <c r="G11" s="9" t="inlineStr">
+      <c r="G11" s="24" t="inlineStr">
         <is>
           <t>PRD v1 §13 Risks/Mitigations</t>
         </is>
@@ -3982,12 +3982,12 @@
           <t>Template Detection (Cross-Author)</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>Optional PubMedBERT / SciSpaCy NER enrichment</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C13" s="24" t="inlineStr">
         <is>
           <t>Model-based biomedical NER can supplement the regex masking layer; default confidence threshold 0.80. Explicitly optional.</t>
         </is>
@@ -4002,12 +4002,12 @@
           <t>Keep</t>
         </is>
       </c>
-      <c r="F13" s="9" t="inlineStr">
+      <c r="F13" s="24" t="inlineStr">
         <is>
           <t>Genuinely additive and non-blocking. Document graceful degradation to regex-only when the model is unavailable or times out -- current behaviour on model failure is unspecified.</t>
         </is>
       </c>
-      <c r="G13" s="9" t="inlineStr">
+      <c r="G13" s="24" t="inlineStr">
         <is>
           <t>Template Detection §4</t>
         </is>
@@ -4066,12 +4066,12 @@
           <t>Template Detection (Cross-Author)</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="24" t="inlineStr">
         <is>
           <t>Direct-Text-Reuse Detector (SequenceMatcher + generic-phrase filtering + corpus-aware distinctive sentences)</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="24" t="inlineStr">
         <is>
           <t>difflib.SequenceMatcher on word tokens, with generic-boilerplate filtering and a corpus-frequency check so rare shared sentences count more than common ones.</t>
         </is>
@@ -4086,12 +4086,12 @@
           <t>Keep</t>
         </is>
       </c>
-      <c r="F15" s="9" t="inlineStr">
+      <c r="F15" s="24" t="inlineStr">
         <is>
           <t>No behavioural change needed. difflib.SequenceMatcher is O(n·m); benchmark against rapidfuzz as a drop-in if runtime becomes an issue at scale.</t>
         </is>
       </c>
-      <c r="G15" s="9" t="inlineStr">
+      <c r="G15" s="24" t="inlineStr">
         <is>
           <t>Template Detection §6</t>
         </is>
@@ -4150,12 +4150,12 @@
           <t>Template Detection (Cross-Author)</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="24" t="inlineStr">
         <is>
           <t>Evidence Combination (primary = strongest signal, not summed; supporting adds ≤0.25)</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="24" t="inlineStr">
         <is>
           <t>Multiple primary signals are not additive -- the strongest one is used; supporting evidence can only nudge the score, never create a finding alone.</t>
         </is>
@@ -4170,12 +4170,12 @@
           <t>Keep</t>
         </is>
       </c>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="F17" s="24" t="inlineStr">
         <is>
           <t>No change. This correctly prevents several mediocre signals from outscoring one real duplicate.</t>
         </is>
       </c>
-      <c r="G17" s="9" t="inlineStr">
+      <c r="G17" s="24" t="inlineStr">
         <is>
           <t>Template Detection §8</t>
         </is>
@@ -4234,12 +4234,12 @@
           <t>Template Detection (Cross-Author)</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t>Template-Family Graph Clustering</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C19" s="24" t="inlineStr">
         <is>
           <t>Template pairs are modeled as graph edges; connected components of ≥3 abstracts can be identified as families -- fully built, explicitly 'not surfaced to editors.'</t>
         </is>
@@ -4254,12 +4254,12 @@
           <t>Keep</t>
         </is>
       </c>
-      <c r="F19" s="9" t="inlineStr">
+      <c r="F19" s="24" t="inlineStr">
         <is>
           <t>Prune-or-ship decision: either add a minimal Template Family view (a 5-abstract family is a much stronger signal than 5 separate pair rows) or delete the code path to stop paying its maintenance cost.</t>
         </is>
       </c>
-      <c r="G19" s="9" t="inlineStr">
+      <c r="G19" s="24" t="inlineStr">
         <is>
           <t>Template Detection §12</t>
         </is>
@@ -4323,12 +4323,12 @@
           <t>LLM Response Trace</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>Known-Pattern Regex Catalogue (YAML rules)</t>
         </is>
       </c>
-      <c r="C21" s="9" t="inlineStr">
+      <c r="C21" s="24" t="inlineStr">
         <is>
           <t>Known LLM-residue phrases live in a YAML rule file matched with Python re, separable from code changes.</t>
         </is>
@@ -4343,12 +4343,12 @@
           <t>Keep</t>
         </is>
       </c>
-      <c r="F21" s="9" t="inlineStr">
+      <c r="F21" s="24" t="inlineStr">
         <is>
           <t>Good practice -- externalized, versionable rules. Recommend the Design Contradiction detector adopt the same YAML pattern (it currently hardcodes its rule table in Python).</t>
         </is>
       </c>
-      <c r="G21" s="9" t="inlineStr">
+      <c r="G21" s="24" t="inlineStr">
         <is>
           <t>LLM Response Trace §3</t>
         </is>
@@ -4407,12 +4407,12 @@
           <t>LLM Response Trace</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="24" t="inlineStr">
         <is>
           <t>Evidence Verification (LLM phrase must literal-match source exactly once)</t>
         </is>
       </c>
-      <c r="C23" s="9" t="inlineStr">
+      <c r="C23" s="24" t="inlineStr">
         <is>
           <t>Any phrase GPT-OSS reports is re-searched in the original preserved text; 0 or &gt;1 matches reject the finding, exactly 1 match restores the exact source characters.</t>
         </is>
@@ -4427,12 +4427,12 @@
           <t>Keep</t>
         </is>
       </c>
-      <c r="F23" s="9" t="inlineStr">
+      <c r="F23" s="24" t="inlineStr">
         <is>
           <t>Excellent anti-hallucination guardrail. Use this exact pattern as the template for the equivalent check already present in Tortured Phrase discovery (§20) -- keep both aligned as the catalogue evolves.</t>
         </is>
       </c>
-      <c r="G23" s="9" t="inlineStr">
+      <c r="G23" s="24" t="inlineStr">
         <is>
           <t>LLM Response Trace §5</t>
         </is>
@@ -4491,12 +4491,12 @@
           <t>LLM Response Trace</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B25" s="24" t="inlineStr">
         <is>
           <t>Context Extraction (quote / blockquote / code-block detection)</t>
         </is>
       </c>
-      <c r="C25" s="9" t="inlineStr">
+      <c r="C25" s="24" t="inlineStr">
         <is>
           <t>Deterministic Python regex/string rules extract the surrounding sentence and detect whether a match sits inside quoted or fenced text.</t>
         </is>
@@ -4511,12 +4511,12 @@
           <t>Enhance</t>
         </is>
       </c>
-      <c r="F25" s="9" t="inlineStr">
+      <c r="F25" s="24" t="inlineStr">
         <is>
           <t>Brittle against smart/curly quotes, nested quotes, or quotes spanning multiple sentences. Normalize Unicode quote characters before detection.</t>
         </is>
       </c>
-      <c r="G25" s="9" t="inlineStr">
+      <c r="G25" s="24" t="inlineStr">
         <is>
           <t>LLM Response Trace §7</t>
         </is>
@@ -4575,12 +4575,12 @@
           <t>LLM Response Trace</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="24" t="inlineStr">
         <is>
           <t>Rule-Based Review Priority (no probability score, no ML weighting)</t>
         </is>
       </c>
-      <c r="C27" s="9" t="inlineStr">
+      <c r="C27" s="24" t="inlineStr">
         <is>
           <t>Priority (High/Medium/Low/none) comes from an explicit lookup table of evidence type, not a trained or weighted model.</t>
         </is>
@@ -4595,12 +4595,12 @@
           <t>Keep</t>
         </is>
       </c>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="F27" s="24" t="inlineStr">
         <is>
           <t>Appropriately explainable for an editorial-trust context; no change needed.</t>
         </is>
       </c>
-      <c r="G27" s="9" t="inlineStr">
+      <c r="G27" s="24" t="inlineStr">
         <is>
           <t>LLM Response Trace §9</t>
         </is>
@@ -4659,12 +4659,12 @@
           <t>Tortured Phrase Detection</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B29" s="24" t="inlineStr">
         <is>
           <t>Regex Phrase Matcher (incl. wildcard prefix, punctuation tolerance, word-boundary guards)</t>
         </is>
       </c>
-      <c r="C29" s="9" t="inlineStr">
+      <c r="C29" s="24" t="inlineStr">
         <is>
           <t>Full regex match after candidate retrieval; tolerates punctuation/whitespace variants, blocks cross-sentence matches, supports `mechan*`-style prefix wildcards.</t>
         </is>
@@ -4679,12 +4679,12 @@
           <t>Enhance</t>
         </is>
       </c>
-      <c r="F29" s="9" t="inlineStr">
+      <c r="F29" s="24" t="inlineStr">
         <is>
           <t>Solid overall, but the dictionary's `~5` proximity operator is parsed and then silently discarded rather than enforced or rejected -- fix or fail loudly at rule-load time.</t>
         </is>
       </c>
-      <c r="G29" s="9" t="inlineStr">
+      <c r="G29" s="24" t="inlineStr">
         <is>
           <t>Tortured Phrase §6-8, §10</t>
         </is>
@@ -4743,12 +4743,12 @@
           <t>Tortured Phrase Detection</t>
         </is>
       </c>
-      <c r="B31" s="9" t="inlineStr">
+      <c r="B31" s="24" t="inlineStr">
         <is>
           <t>Mandatory GPT-OSS Validation (temperature=0) for Known-Phrase Candidates</t>
         </is>
       </c>
-      <c r="C31" s="9" t="inlineStr">
+      <c r="C31" s="24" t="inlineStr">
         <is>
           <t>Every deterministic tortured-phrase match is validated by GPT-OSS with matched phrase, expected term, and surrounding context before it becomes a finding.</t>
         </is>
@@ -4763,12 +4763,12 @@
           <t>Keep</t>
         </is>
       </c>
-      <c r="F31" s="9" t="inlineStr">
+      <c r="F31" s="24" t="inlineStr">
         <is>
           <t>No change needed. Correctly gates the result, matching LLM Response Trace's pattern.</t>
         </is>
       </c>
-      <c r="G31" s="9" t="inlineStr">
+      <c r="G31" s="24" t="inlineStr">
         <is>
           <t>Tortured Phrase §13</t>
         </is>
@@ -4827,12 +4827,12 @@
           <t>Tortured Phrase Detection</t>
         </is>
       </c>
-      <c r="B33" s="9" t="inlineStr">
+      <c r="B33" s="24" t="inlineStr">
         <is>
           <t>Fixed New-Phrase Confidence Mapping (low/med/high → 0.55/0.72/0.88)</t>
         </is>
       </c>
-      <c r="C33" s="9" t="inlineStr">
+      <c r="C33" s="24" t="inlineStr">
         <is>
           <t>GPT-OSS's qualitative confidence is mapped to three fixed numeric values; not calibrated probabilities.</t>
         </is>
@@ -4847,12 +4847,12 @@
           <t>Enhance</t>
         </is>
       </c>
-      <c r="F33" s="9" t="inlineStr">
+      <c r="F33" s="24" t="inlineStr">
         <is>
           <t>Reasonable placeholder; once enough editor accept/reject history exists, recalibrate these three buckets empirically rather than leaving them as guesses.</t>
         </is>
       </c>
-      <c r="G33" s="9" t="inlineStr">
+      <c r="G33" s="24" t="inlineStr">
         <is>
           <t>Tortured Phrase §21</t>
         </is>
@@ -4911,12 +4911,12 @@
           <t>Numerical Contradiction</t>
         </is>
       </c>
-      <c r="B35" s="9" t="inlineStr">
+      <c r="B35" s="24" t="inlineStr">
         <is>
           <t>Numerical Claim Extraction Regex Suite (counts, percentages, medians/ranges, exclusive subgroups)</t>
         </is>
       </c>
-      <c r="C35" s="9" t="inlineStr">
+      <c r="C35" s="24" t="inlineStr">
         <is>
           <t>Regex extracts structured NumericalClaim objects for n/N, percentages, median±range, and explicitly-flagged mutually-exclusive subgroup sums.</t>
         </is>
@@ -4931,12 +4931,12 @@
           <t>Enhance</t>
         </is>
       </c>
-      <c r="F35" s="9" t="inlineStr">
+      <c r="F35" s="24" t="inlineStr">
         <is>
           <t>Solid extraction, but by design it is sentence-local only (see next row) -- the extraction layer itself is fine and doesn't need rework.</t>
         </is>
       </c>
-      <c r="G35" s="9" t="inlineStr">
+      <c r="G35" s="24" t="inlineStr">
         <is>
           <t>Numerical §3-4</t>
         </is>
@@ -4995,12 +4995,12 @@
           <t>Numerical Contradiction</t>
         </is>
       </c>
-      <c r="B37" s="9" t="inlineStr">
+      <c r="B37" s="24" t="inlineStr">
         <is>
           <t>Arithmetic / Boundary Rule Engine (mismatch, exceeds-N, impossible %, median-outside-range, reversed interval, exclusive-group overrun)</t>
         </is>
       </c>
-      <c r="C37" s="9" t="inlineStr">
+      <c r="C37" s="24" t="inlineStr">
         <is>
           <t>Six explicit deterministic rules with fixed thresholds (e.g. 1.0 percentage-point tolerance) directly test extracted claims.</t>
         </is>
@@ -5015,12 +5015,12 @@
           <t>Keep</t>
         </is>
       </c>
-      <c r="F37" s="9" t="inlineStr">
+      <c r="F37" s="24" t="inlineStr">
         <is>
           <t>Sound and appropriately conservative. No change needed beyond moving the tolerance constant into shared config (see P2 row).</t>
         </is>
       </c>
-      <c r="G37" s="9" t="inlineStr">
+      <c r="G37" s="24" t="inlineStr">
         <is>
           <t>Numerical §5</t>
         </is>
@@ -5079,12 +5079,12 @@
           <t>Numerical Contradiction</t>
         </is>
       </c>
-      <c r="B39" s="9" t="inlineStr">
+      <c r="B39" s="24" t="inlineStr">
         <is>
           <t>Relative-Percentage Guard (&gt;100% is not automatically impossible)</t>
         </is>
       </c>
-      <c r="C39" s="9" t="inlineStr">
+      <c r="C39" s="24" t="inlineStr">
         <is>
           <t>Nearby text is checked for relative-change language (increase, reduction, dose intensity) before a &gt;100% value is treated as an impossible absolute rate.</t>
         </is>
@@ -5099,12 +5099,12 @@
           <t>Keep</t>
         </is>
       </c>
-      <c r="F39" s="9" t="inlineStr">
+      <c r="F39" s="24" t="inlineStr">
         <is>
           <t>No change needed -- a genuinely good false-positive guard.</t>
         </is>
       </c>
-      <c r="G39" s="9" t="inlineStr">
+      <c r="G39" s="24" t="inlineStr">
         <is>
           <t>Numerical §6</t>
         </is>
@@ -5163,12 +5163,12 @@
           <t>Design Contradiction</t>
         </is>
       </c>
-      <c r="B41" s="9" t="inlineStr">
+      <c r="B41" s="24" t="inlineStr">
         <is>
           <t>Future-Work Statement Guard</t>
         </is>
       </c>
-      <c r="C41" s="9" t="inlineStr">
+      <c r="C41" s="24" t="inlineStr">
         <is>
           <t>Prospective/randomized/blinded phrases are ignored when the sentence is clearly describing proposed or future work ('future prospective trials are required').</t>
         </is>
@@ -5183,12 +5183,12 @@
           <t>Keep</t>
         </is>
       </c>
-      <c r="F41" s="9" t="inlineStr">
+      <c r="F41" s="24" t="inlineStr">
         <is>
           <t>Well-reasoned guard; no change needed.</t>
         </is>
       </c>
-      <c r="G41" s="9" t="inlineStr">
+      <c r="G41" s="24" t="inlineStr">
         <is>
           <t>Numerical/Design/Trial §12</t>
         </is>
@@ -5247,12 +5247,12 @@
           <t>Design Contradiction</t>
         </is>
       </c>
-      <c r="B43" s="9" t="inlineStr">
+      <c r="B43" s="24" t="inlineStr">
         <is>
           <t>Pairwise Contradiction Rule Table (fixed ~9 incompatible-value pairs via itertools.combinations)</t>
         </is>
       </c>
-      <c r="C43" s="9" t="inlineStr">
+      <c r="C43" s="24" t="inlineStr">
         <is>
           <t>Every pair of extracted claims within a record is tested against a closed table of incompatible design-value pairs.</t>
         </is>
@@ -5267,12 +5267,12 @@
           <t>Enhance</t>
         </is>
       </c>
-      <c r="F43" s="9" t="inlineStr">
+      <c r="F43" s="24" t="inlineStr">
         <is>
           <t>Combinatorics are not a scale risk here (few claims per abstract). The risk is a closed rule list: new contradiction types require a code change, not a data change.</t>
         </is>
       </c>
-      <c r="G43" s="9" t="inlineStr">
+      <c r="G43" s="24" t="inlineStr">
         <is>
           <t>Numerical/Design/Trial §13</t>
         </is>
@@ -5331,12 +5331,12 @@
           <t>Design Contradiction</t>
         </is>
       </c>
-      <c r="B45" s="9" t="inlineStr">
+      <c r="B45" s="24" t="inlineStr">
         <is>
           <t>Legitimate-Mixed-Design Exception List (10+ named patterns)</t>
         </is>
       </c>
-      <c r="C45" s="9" t="inlineStr">
+      <c r="C45" s="24" t="inlineStr">
         <is>
           <t>Specific, named exceptions (retrospective analysis of an RCT, open-label extension after blinded period, phase II/III seamless design, etc.) suppress known-legitimate contradictions.</t>
         </is>
@@ -5351,12 +5351,12 @@
           <t>Enhance</t>
         </is>
       </c>
-      <c r="F45" s="9" t="inlineStr">
+      <c r="F45" s="24" t="inlineStr">
         <is>
           <t>Reasonable for V1; same closed-list drift risk as the rule table above. Establish a periodic review cadence as new legitimate design patterns are encountered.</t>
         </is>
       </c>
-      <c r="G45" s="9" t="inlineStr">
+      <c r="G45" s="24" t="inlineStr">
         <is>
           <t>Numerical/Design/Trial §14</t>
         </is>
@@ -5415,12 +5415,12 @@
           <t>Unverifiable Clinical Trial</t>
         </is>
       </c>
-      <c r="B47" s="9" t="inlineStr">
+      <c r="B47" s="24" t="inlineStr">
         <is>
           <t>Registry-ID / Registration-Phrase Regex Extraction</t>
         </is>
       </c>
-      <c r="C47" s="9" t="inlineStr">
+      <c r="C47" s="24" t="inlineStr">
         <is>
           <t>Deliberately permissive regexes extract NCT/ISRCTN/ACTRN/EUCTR/EudraCT/ChiCTR references plus placeholder ('pending', 'TBD') and no-ID registration claims.</t>
         </is>
@@ -5435,12 +5435,12 @@
           <t>Enhance</t>
         </is>
       </c>
-      <c r="F47" s="9" t="inlineStr">
+      <c r="F47" s="24" t="inlineStr">
         <is>
           <t>Supported-registry list omits several registries in active global use (India's CTRI, Germany's DRKS, Japan's jRCT, Iran's IRCT). For an internationally-submitted corpus this is a real, if low-severity, coverage gap.</t>
         </is>
       </c>
-      <c r="G47" s="9" t="inlineStr">
+      <c r="G47" s="24" t="inlineStr">
         <is>
           <t>Numerical/Design/Trial §19</t>
         </is>
@@ -5504,12 +5504,12 @@
           <t>Unverifiable Clinical Trial</t>
         </is>
       </c>
-      <c r="B49" s="9" t="inlineStr">
+      <c r="B49" s="24" t="inlineStr">
         <is>
           <t>Local Classification (placeholder / no-ID / malformed / unsupported registry)</t>
         </is>
       </c>
-      <c r="C49" s="9" t="inlineStr">
+      <c r="C49" s="24" t="inlineStr">
         <is>
           <t>Claims that don't need a network call are classified deterministically without ever reaching the registry adapter.</t>
         </is>
@@ -5524,12 +5524,12 @@
           <t>Keep</t>
         </is>
       </c>
-      <c r="F49" s="9" t="inlineStr">
+      <c r="F49" s="24" t="inlineStr">
         <is>
           <t>No change needed -- correct separation of concerns between local classification and authoritative lookup.</t>
         </is>
       </c>
-      <c r="G49" s="9" t="inlineStr">
+      <c r="G49" s="24" t="inlineStr">
         <is>
           <t>Numerical/Design/Trial §21</t>
         </is>
@@ -5588,12 +5588,12 @@
           <t>Unverifiable Clinical Trial</t>
         </is>
       </c>
-      <c r="B51" s="9" t="inlineStr">
+      <c r="B51" s="24" t="inlineStr">
         <is>
           <t>Registry-Result Self-Consistency Validation</t>
         </is>
       </c>
-      <c r="C51" s="9" t="inlineStr">
+      <c r="C51" s="24" t="inlineStr">
         <is>
           <t>Returned adapter objects are checked for registry-name match, ID match, found/verified consistency, and correct external-ID echoing before being trusted.</t>
         </is>
@@ -5608,12 +5608,12 @@
           <t>Keep</t>
         </is>
       </c>
-      <c r="F51" s="9" t="inlineStr">
+      <c r="F51" s="24" t="inlineStr">
         <is>
           <t>Excellent defensive check against a malformed or mismatched adapter response; no change needed.</t>
         </is>
       </c>
-      <c r="G51" s="9" t="inlineStr">
+      <c r="G51" s="24" t="inlineStr">
         <is>
           <t>Numerical/Design/Trial §23</t>
         </is>
@@ -5672,12 +5672,12 @@
           <t>Unverifiable Clinical Trial</t>
         </is>
       </c>
-      <c r="B53" s="9" t="inlineStr">
+      <c r="B53" s="24" t="inlineStr">
         <is>
           <t>`urllib.request` as the HTTP Layer</t>
         </is>
       </c>
-      <c r="C53" s="9" t="inlineStr">
+      <c r="C53" s="24" t="inlineStr">
         <is>
           <t>Standard-library urllib is used directly rather than a session-based HTTP client.</t>
         </is>
@@ -5692,12 +5692,12 @@
           <t>Enhance</t>
         </is>
       </c>
-      <c r="F53" s="9" t="inlineStr">
+      <c r="F53" s="24" t="inlineStr">
         <is>
           <t>Current behavior is documented and correct; low-priority swap to `requests`/`httpx` with a pooled session would reduce hand-rolled edge-case surface (redirects, TLS, charset) on any future touch of this module.</t>
         </is>
       </c>
-      <c r="G53" s="9" t="inlineStr">
+      <c r="G53" s="24" t="inlineStr">
         <is>
           <t>Numerical/Design/Trial §22</t>
         </is>
@@ -5756,12 +5756,12 @@
           <t>Consolidated Workbook / Reporting</t>
         </is>
       </c>
-      <c r="B55" s="9" t="inlineStr">
+      <c r="B55" s="24" t="inlineStr">
         <is>
           <t>Check Detail Sheet (evidence pointer, not raw text)</t>
         </is>
       </c>
-      <c r="C55" s="9" t="inlineStr">
+      <c r="C55" s="24" t="inlineStr">
         <is>
           <t>Consolidated sheet stays scannable by referring to 'See Template Evidence (N pair(s))' rather than embedding large comparison text inline.</t>
         </is>
@@ -5776,12 +5776,12 @@
           <t>Keep</t>
         </is>
       </c>
-      <c r="F55" s="9" t="inlineStr">
+      <c r="F55" s="24" t="inlineStr">
         <is>
           <t>Good UX decision -- keeps the master sheet usable at scale. No change needed.</t>
         </is>
       </c>
-      <c r="G55" s="9" t="inlineStr">
+      <c r="G55" s="24" t="inlineStr">
         <is>
           <t>Template Detection §13</t>
         </is>
@@ -5840,12 +5840,12 @@
           <t>Consolidated Workbook / Reporting</t>
         </is>
       </c>
-      <c r="B57" s="9" t="inlineStr">
+      <c r="B57" s="24" t="inlineStr">
         <is>
           <t>Structured-Field Export (numeric deltas, trial registry metadata, design validation reason)</t>
         </is>
       </c>
-      <c r="C57" s="9" t="inlineStr">
+      <c r="C57" s="24" t="inlineStr">
         <is>
           <t>Detectors internally compute calculated_value/difference/tolerance (numerical), registry phase/conditions/interventions (trial), and validation_status/reason (design) -- none currently reach the exported workbook/UI.</t>
         </is>
@@ -5860,12 +5860,12 @@
           <t>Enhance</t>
         </is>
       </c>
-      <c r="F57" s="9" t="inlineStr">
+      <c r="F57" s="24" t="inlineStr">
         <is>
           <t>Near-zero-cost win: these fields are already computed. Expose them as additional (optionally collapsed) columns instead of leaving them stranded in the native detector output.</t>
         </is>
       </c>
-      <c r="G57" s="9" t="inlineStr">
+      <c r="G57" s="24" t="inlineStr">
         <is>
           <t>Numerical/Design/Trial §9, §17, §27</t>
         </is>
@@ -5929,12 +5929,12 @@
           <t>Editor Frontend &amp; Evals</t>
         </is>
       </c>
-      <c r="B59" s="9" t="inlineStr">
+      <c r="B59" s="24" t="inlineStr">
         <is>
           <t>Submission Detail View (per-check flagged/evidence display)</t>
         </is>
       </c>
-      <c r="C59" s="9" t="inlineStr">
+      <c r="C59" s="24" t="inlineStr">
         <is>
           <t>React UI shows flagged status, match count, and concatenated plain-English evidence per check on the submission detail screen.</t>
         </is>
@@ -5949,12 +5949,12 @@
           <t>Keep</t>
         </is>
       </c>
-      <c r="F59" s="9" t="inlineStr">
+      <c r="F59" s="24" t="inlineStr">
         <is>
           <t>No change needed.</t>
         </is>
       </c>
-      <c r="G59" s="9" t="inlineStr">
+      <c r="G59" s="24" t="inlineStr">
         <is>
           <t>Numerical/Design/Trial §28</t>
         </is>
@@ -6013,12 +6013,12 @@
           <t>Editor Frontend &amp; Evals</t>
         </is>
       </c>
-      <c r="B61" s="9" t="inlineStr">
+      <c r="B61" s="24" t="inlineStr">
         <is>
           <t>Evals View (validation results for 2 of 3 LLM-validated checks)</t>
         </is>
       </c>
-      <c r="C61" s="9" t="inlineStr">
+      <c r="C61" s="24" t="inlineStr">
         <is>
           <t>Dedicated view for reviewing GPT-OSS validation outcomes currently covers Tortured Phrase and LLM Response Trace only.</t>
         </is>
@@ -6033,12 +6033,12 @@
           <t>Enhance</t>
         </is>
       </c>
-      <c r="F61" s="9" t="inlineStr">
+      <c r="F61" s="24" t="inlineStr">
         <is>
           <t>Once Design Contradiction's validation is wired to gate its flag (P7 fix), extend Evals to cover it too, for consistency across all three LLM-validated checks.</t>
         </is>
       </c>
-      <c r="G61" s="9" t="inlineStr">
+      <c r="G61" s="24" t="inlineStr">
         <is>
           <t>Numerical/Design/Trial §17, §29</t>
         </is>
@@ -7068,42 +7068,42 @@
       </c>
     </row>
     <row r="2" ht="24" customHeight="1" s="22">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>Issue ID</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="23" t="inlineStr">
         <is>
           <t>Pipeline(s) Affected</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="23" t="inlineStr">
         <is>
           <t>Pattern Type</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="23" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="23" t="inlineStr">
         <is>
           <t>Real-World Failure Scenario</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="23" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="23" t="inlineStr">
         <is>
           <t>Recommended Fix</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="23" t="inlineStr">
         <is>
           <t>Roadmap Phase</t>
         </is>
@@ -7120,7 +7120,7 @@
           <t>OE-01</t>
         </is>
       </c>
-      <c r="B3" s="9" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>XML Ingestion &amp; Record Parsing; Numerical Contradiction; Design Contradiction; Unverifiable Clinical Trial</t>
         </is>
@@ -7130,12 +7130,12 @@
           <t>Duplicated Logic</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="24" t="inlineStr">
         <is>
           <t>The naive sentence splitter regex (?&lt;=[.!?])\s+ is independently reimplemented in at least three detector modules instead of living in one shared utility.</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="24" t="inlineStr">
         <is>
           <t>Common biomedical abbreviations (Fig., vs., e.g., no., i.v.) and decimal-adjacent punctuation fracture sentences, corrupting numeric-claim boundaries and the exact-context windows sent to GPT-OSS -- and any future fix has to be applied N times, not once.</t>
         </is>
@@ -7145,7 +7145,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="G3" s="24" t="inlineStr">
         <is>
           <t>Extract one shared sentence_split() utility using an abbreviation-aware tokenizer (pySBD or a spaCy rule-based sentencizer); delete every per-module copy.</t>
         </is>
@@ -7202,6 +7202,11 @@
           <t>Phase 2</t>
         </is>
       </c>
+      <c r="I4" s="24" t="inlineStr">
+        <is>
+          <t>Resolved — Phase 2 (2026-08-19). Added warning at tortured-phrase dictionary-load time (load_tortured_rules) when ~N proximity operator appears on single-token rules (unsupported; proximity matching requires 2+ tokens). Rule authors now see explicit stacklevel=2 warning instead of silent discard, closing the gap between perceived and actual rule behavior.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="79.5" customHeight="1" s="22">
       <c r="A5" s="7" t="inlineStr">
@@ -7209,7 +7214,7 @@
           <t>OE-03</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Design Contradiction</t>
         </is>
@@ -7219,12 +7224,12 @@
           <t>Over-Engineered (dead compute) / Inconsistent Behavior</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="24" t="inlineStr">
         <is>
           <t>GPT-OSS validates every design-contradiction candidate, but a rejected result never suppresses the finding -- it is stored as an annotation while check_triggered stays True.</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="24" t="inlineStr">
         <is>
           <t>An editor can see an active 'contradiction found' flag sitting directly next to an internally-stored 'rejected' reason. The first time someone notices this, trust in every other check erodes -- and today the org pays LLM latency/cost for a signal that structurally cannot change the outcome.</t>
         </is>
@@ -7234,7 +7239,7 @@
           <t>Critical</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="G5" s="24" t="inlineStr">
         <is>
           <t>Gate the flag on validation_status exactly as Tortured Phrase and LLM Response Trace already do (confirmed/rejected/uncertain controls the active result).</t>
         </is>
@@ -7242,6 +7247,11 @@
       <c r="H5" s="7" t="inlineStr">
         <is>
           <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="I5" s="24" t="inlineStr">
+        <is>
+          <t>Resolved — Phase 2 (2026-08-19). Design contradiction findings now gate check_triggered on validation_status exactly as tortured_phrase and llm_response_trace do: when GPT-OSS validation returns 'rejected', the finding is marked check_triggered=False, making it inactive so it no longer displays as flagged. Verified by new test: test_rejected_validation_deactivates_detected_contradiction.</t>
         </is>
       </c>
     </row>
@@ -7293,7 +7303,7 @@
           <t>OE-05</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>Template Detection (Cross-Author)</t>
         </is>
@@ -7303,12 +7313,12 @@
           <t>Dead / Orphaned Capability</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="24" t="inlineStr">
         <is>
           <t>Connected-component clustering of template families (≥3 linked abstracts) is fully implemented as a graph structure but explicitly documented as not surfaced to editors.</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="24" t="inlineStr">
         <is>
           <t>Ongoing maintenance cost for a feature nobody consumes -- and editors reviewing 5 separate pairwise rows for what is actually one 5-abstract templated family never see the single strongest signal the system already computed: family size.</t>
         </is>
@@ -7318,7 +7328,7 @@
           <t>Medium</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="G7" s="24" t="inlineStr">
         <is>
           <t>Ship a minimal Template Family view, or delete the code path. Do not leave a half-built capability as permanent technical debt.</t>
         </is>
@@ -7387,7 +7397,7 @@
           <t>OE-07</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="24" t="inlineStr">
         <is>
           <t>Tortured Phrase Detection; LLM Response Trace; Design Contradiction</t>
         </is>
@@ -7397,12 +7407,12 @@
           <t>Narrow-Brittle (Inconsistent Resilience)</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="24" t="inlineStr">
         <is>
           <t>The ClinicalTrials.gov adapter has explicit timeout/retry/backoff/caching; the three GPT-OSS call sites used across these pipelines document no equivalent resilience pattern.</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="24" t="inlineStr">
         <is>
           <t>A transient IntelliHub rate-limit or outage during a ~6,000-abstract run can silently degrade or fail an unknown number of tortured-phrase / LLM-trace / design-contradiction validations, with none of the retry/backoff discipline the registry lookups already have.</t>
         </is>
@@ -7412,7 +7422,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="G9" s="24" t="inlineStr">
         <is>
           <t>One shared LLM client wrapper with the same timeout/retry/backoff/cache discipline as the registry adapter, used uniformly by all three call sites.</t>
         </is>
@@ -7476,7 +7486,7 @@
           <t>OE-09</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Numerical Contradiction</t>
         </is>
@@ -7486,12 +7496,12 @@
           <t>Narrow Solution (Documented V1 Gap)</t>
         </is>
       </c>
-      <c r="D11" s="9" t="inlineStr">
+      <c r="D11" s="24" t="inlineStr">
         <is>
           <t>The detector cannot connect a population count stated in one sentence to a percentage or count stated in a later sentence -- explicitly acknowledged as sentence-local-only in the design doc.</t>
         </is>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E11" s="24" t="inlineStr">
         <is>
           <t>The single most common numeric-contradiction pattern in real abstracts ('120 patients were enrolled. ... the response rate was 45% (58/110).') is structurally invisible today, because N and the percentage claim live in different sentences.</t>
         </is>
@@ -7501,7 +7511,7 @@
           <t>High</t>
         </is>
       </c>
-      <c r="G11" s="9" t="inlineStr">
+      <c r="G11" s="24" t="inlineStr">
         <is>
           <t>Add a lightweight cross-sentence 'most recently stated N' carry-forward pass ahead of the existing arithmetic rules -- no LLM or embeddings required.</t>
         </is>
@@ -8595,42 +8605,42 @@
       </c>
     </row>
     <row r="2" ht="24" customHeight="1" s="22">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" s="23" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="23" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="23" t="inlineStr">
         <is>
           <t>Target Duration</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="23" t="inlineStr">
         <is>
           <t>Scope / Key Changes</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="23" t="inlineStr">
         <is>
           <t>Rationale</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" s="23" t="inlineStr">
         <is>
           <t>Effort</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="23" t="inlineStr">
         <is>
           <t>Dependencies</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="H2" s="23" t="inlineStr">
         <is>
           <t>Success Criteria</t>
         </is>
@@ -8657,12 +8667,12 @@
           <t>1–2 wks</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="D3" s="24" t="inlineStr">
         <is>
           <t>Add run metadata + dictionary/rule-version stamping visible in the workbook for every rule source (not just tortured phrases); add structured parse-failure and record-exclusion reporting; add latency/success telemetry around every GPT-OSS call site.</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="E3" s="24" t="inlineStr">
         <is>
           <t>You cannot safely refactor a system you can't yet observe. This phase adds guardrails and visibility without changing any detector's behavior, so it de-risks everything that follows.</t>
         </is>
@@ -8672,12 +8682,12 @@
           <t>S</t>
         </is>
       </c>
-      <c r="G3" s="9" t="inlineStr">
+      <c r="G3" s="24" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="H3" s="9" t="inlineStr">
+      <c r="H3" s="24" t="inlineStr">
         <is>
           <t>Every pipeline run produces one run report showing parse failures, rule/dictionary versions, and LLM call success/latency stats.</t>
         </is>
@@ -8751,12 +8761,12 @@
           <t>1–2 wks</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="D5" s="24" t="inlineStr">
         <is>
           <t>Gate the Design Contradiction flag on its own LLM validation_status, matching Tortured Phrase / LLM Response Trace behavior (OE-03); fix or explicitly disable the silently-ignored ~5 proximity operator in the tortured-phrase dictionary (OE-02); replace the binary High/Low risk collapse with the graded priority every detector already computes (OE-10).</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="24" t="inlineStr">
         <is>
           <t>These are the clearest cases where the system's actual behavior silently diverges from what an editor would reasonably assume it does. High trust impact, low engineering cost -- fix before anything more ambitious.</t>
         </is>
@@ -8766,14 +8776,19 @@
           <t>S</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="G5" s="24" t="inlineStr">
         <is>
           <t>Phase 0 telemetry confirms no hidden dependents on current non-gating/binary behavior</t>
         </is>
       </c>
-      <c r="H5" s="9" t="inlineStr">
+      <c r="H5" s="24" t="inlineStr">
         <is>
           <t>All three LLM-validated checks behave identically (confirmed/rejected/uncertain drives the same gating logic); a dictionary rule using ~N either enforces it or fails to load with a clear error; the editor-facing risk badge reflects native per-check severity.</t>
+        </is>
+      </c>
+      <c r="I5" s="24" t="inlineStr">
+        <is>
+          <t>Done — 2026-08-19. OE-03 (CRITICAL) resolved: design_contradiction findings now gate check_triggered on validation_status, deactivating rejected findings. OE-02 resolved: tortured-phrase dictionary-load warns loudly on unsupported ~N single-token proximity. OE-10 verification: graded priority (None/Low/Medium/High) already exists in _risk_from_signals; exported as overall_content_risk in summary. Full test suite green (261 passed) plus 2 new subtest variants on OE-03.</t>
         </is>
       </c>
     </row>
@@ -8835,12 +8850,12 @@
           <t>Ongoing, as volume grows</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
+      <c r="D7" s="24" t="inlineStr">
         <is>
           <t>Introduce ANN/MinHash-LSH candidate generation ahead of Template Detection's deterministic classifiers to remove the pairwise O(n²) ceiling (OE-04); surface currently-computed-but-hidden structured fields (numerical calculated_value/difference, trial registry metadata, design validation reason) in the workbook/UI; calibrate the fixed low/med/high confidence mapping in tortured-phrase discovery against real editor accept/reject history.</t>
         </is>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="24" t="inlineStr">
         <is>
           <t>Unlocks value the system already computes internally and removes the one clear scalability ceiling, without touching the deterministic-first philosophy that gives the system its explainability and editorial trust.</t>
         </is>
@@ -8850,12 +8865,12 @@
           <t>L</t>
         </is>
       </c>
-      <c r="G7" s="9" t="inlineStr">
+      <c r="G7" s="24" t="inlineStr">
         <is>
           <t>Phases 0–2 complete; sufficient review-history data for calibration</t>
         </is>
       </c>
-      <c r="H7" s="9" t="inlineStr">
+      <c r="H7" s="24" t="inlineStr">
         <is>
           <t>Template-detection runtime stays sub-quadratic-feeling as the corpus grows across years; editors report priority badges match their own sense of urgency; zero 'computed but hidden' fields remain undocumented.</t>
         </is>

</xml_diff>

<commit_message>
Correct stale OE-03 workbook notes after check_triggered revert
Overengineering Log OE-03 and Refactoring Roadmap Phase 2 both still
described the reverted check_triggered=False change as the resolution.
Updated both notes to reflect that design_contradiction was already
correctly gated via the shared Finding.active property before Phase 2,
and that the check_triggered change broke that field's contract and
was reverted (ffef2e9).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Content_Integrity_Pipeline_Audit.xlsx
+++ b/Content_Integrity_Pipeline_Audit.xlsx
@@ -7251,7 +7251,7 @@
       </c>
       <c r="I5" s="24" t="inlineStr">
         <is>
-          <t>Resolved — Phase 2 (2026-08-19). Design contradiction findings now gate check_triggered on validation_status exactly as tortured_phrase and llm_response_trace do: when GPT-OSS validation returns 'rejected', the finding is marked check_triggered=False, making it inactive so it no longer displays as flagged. Verified by new test: test_rejected_validation_deactivates_detected_contradiction.</t>
+          <t>Resolved — was already correct before Phase 2 touched it; corrected on verification pass (2026-08-19). The Phase 2 commit (d803b5a) added check_triggered=False on validation_status="rejected", but design_contradiction already gated the display/suppression behavior correctly via the shared Finding.active property (active = validation_status not in INACTIVE_VALIDATION_STATUSES), matching tortured_phrase and llm_response_trace, which do not have a check_triggered field at all. Setting check_triggered=False on rejected broke that field's actual contract (it records that the detector logic fired, independent of validation outcome) and was reverted (ffef2e9). Confirmed downstream consumers (design_contradiction_flag, risk-eligibility filtering in pipeline.py) key off .active, not check_triggered, so rejected findings are correctly suppressed from editor-facing display. Test test_rejected_validation_deactivates_detected_contradiction still passes and now asserts the correct contract: check_triggered stays True, active is False.</t>
         </is>
       </c>
     </row>
@@ -8788,7 +8788,7 @@
       </c>
       <c r="I5" s="24" t="inlineStr">
         <is>
-          <t>Done — 2026-08-19. OE-03 (CRITICAL) resolved: design_contradiction findings now gate check_triggered on validation_status, deactivating rejected findings. OE-02 resolved: tortured-phrase dictionary-load warns loudly on unsupported ~N single-token proximity. OE-10 verification: graded priority (None/Low/Medium/High) already exists in _risk_from_signals; exported as overall_content_risk in summary. Full test suite green (261 passed) plus 2 new subtest variants on OE-03.</t>
+          <t>Done — 2026-08-19, corrected on verification pass (2026-08-19). OE-03 (CRITICAL): design_contradiction was already correctly gated via the shared Finding.active property before Phase 2; the check_triggered=False change this phase added broke that field's contract and was reverted (ffef2e9) — see Overengineering Log OE-03 for detail. OE-02 resolved, with a follow-up fix on verification: tortured-phrase dictionary-load now warns on unsupported ~N single-token proximity for the common bare-rule case too (the original Phase 2 fix only warned when the single-token rule also had an AND/NOT clause). OE-10 verification: graded priority (None/Low/Medium/High) already exists in _risk_from_signals; exported as overall_content_risk in summary. Full test suite green (264 passed) plus subtest variants on OE-03, apart from one pre-existing, unrelated authorship-reporting failure.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update audit workbook for Phase 3: OE-07, OE-08, OE-09 resolved
Reflects the actual work: OE-09's conservative cross-sentence carry-
forward, OE-07's finding that timeout/retry/backoff was already shared
across all three GPT-OSS call sites (only caching was genuinely
missing), and OE-08's registry expansion plus the WHO-ICTRP hyphen bug
caught during that work. Also notes the untracked-test-fixture gap
found by two of the three parallel workstreams.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Content_Integrity_Pipeline_Audit.xlsx
+++ b/Content_Integrity_Pipeline_Audit.xlsx
@@ -7432,6 +7432,11 @@
           <t>Phase 3</t>
         </is>
       </c>
+      <c r="I9" s="0" t="inlineStr">
+        <is>
+          <t>Resolved — 2026-08-20. Verified first: the shared IntelliHubGPTOSSClient (all three GPT-OSS call sites — tortured_phrase/llm_response_trace via ContextValidator, design_contradiction via LLMDesignContradictionValidator, llm_response_trace via LLMTraceValidator — already route through one client instance built once in pipeline.py) already had per-request timeout, retry with exponential backoff on HTTP 429/5xx, and CallStats telemetry, apparently added during Phase 0 instrumentation but never credited against this row. The one genuine gap versus ClinicalTrialsGovClient — no caching — is now closed: content-addressed persistent JSON caching (sha256 of endpoint+full payload, one file per key, cache_dir=None default = off, matching the registry client's off-by-default pattern), wired via config.output_dir/".gpt_oss_cache". Verified by new tests/test_context_validator.py (cache miss writes + calls live, cache hit skips the network call and leaves CallStats untouched, different payloads never collide, caching-off is unchanged behavior).</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="79.5" customHeight="1" s="22">
       <c r="A10" s="10" t="inlineStr">
@@ -7476,7 +7481,7 @@
       </c>
       <c r="I10" s="24" t="inlineStr">
         <is>
-          <t>Partially resolved — Phase 1 (2026-08-19). The 'three separately-maintained vocabulary copies' claim did not hold on inspection: template_matching_common.py already exists as one shared module for gene/drug/trial-ID patterns, reused by entity_extraction.py, entity_normalized_template.py, and unverifiable_trial.py; tortured_phrase.py has no vocabulary at all (it loads an unrelated CSV phrase dictionary). The genuine duplication found — the trial-registry prefix list hand-typed 4 times in/around unverifiable_trial.py — is now built from one SUPPORTED_REGISTRY_PREFIXES tuple, with an assertion keeping REGISTRY_NAMES in sync. Registry coverage itself (CTRI/DRKS/jRCT/IRCT/WHO ICTRP) is unchanged and remains Phase 3.</t>
+          <t>Resolved — Phase 1 vocabulary consolidation (2026-08-19), registry coverage completed Phase 3 (2026-08-20). The 'three separately-maintained vocabulary copies' claim did not hold on inspection: template_matching_common.py already exists as one shared module for gene/drug/trial-ID patterns; tortured_phrase.py has no vocabulary at all. The genuine duplication found — the trial-registry prefix list hand-typed 4 times — is now built from one SUPPORTED_REGISTRY_PREFIXES tuple with an assertion keeping REGISTRY_NAMES in sync. Registry coverage now added: CTRI, DRKS, jRCT, IRCT, and WHO ICTRP's Universal Trial Number, format-validation-only (no live API — same tier as the 5 pre-existing non-NCT registries; only ClinicalTrials.gov has a live lookup client). Caught and fixed a real bug in the same pass: OTHER_REGISTRY_RE's optional separator group would have silently eaten the mandatory hyphen in every WHO ICTRP UTN (U1111-XXXX-XXXX), corrupting the normalized id and failing every real UTN's format check; U1111 now routes through the separator-free TRIAL_PATTERN fallback instead. Confidence varies by registry — CTRI and DRKS formats are well-documented and high-confidence; jRCT (least standardized registry format of the five, multiple sub-registry code variants) and the WHO ICTRP UTN (real-world prevalence in abstract text as a meta-registry aggregator, not a primary registration) are lower-confidence and worth spot-checking against real submissions if this flags unexpectedly. Verified by new tests in tests/test_unverifiable_trial.py: format validation (valid/invalid) and sentence extraction for all 5 new registries.</t>
         </is>
       </c>
     </row>
@@ -7519,6 +7524,11 @@
       <c r="H11" s="7" t="inlineStr">
         <is>
           <t>Phase 3</t>
+        </is>
+      </c>
+      <c r="I11" s="0" t="inlineStr">
+        <is>
+          <t>Resolved — 2026-08-20. Added a lightweight cross-sentence carry-forward pass to numerical_contradiction.py exactly as the Recommended Fix describes (no LLM/embeddings). The most recently stated population total ("120 patients were enrolled", "among 120 patients") is tracked per record in document order and used as the denominator for a later percentage/count claim that states no local denominator, gated by population-noun agreement and a DIFFERENT_POPULATION_RE guard (evaluable/eligible/responders/named subgroup/etc.) applied both when updating the carried total and when linking a later claim, so a subset count never leaks forward as the whole population and a differently-qualified later claim never gets linked to an unrelated total. Carried-forward findings get their own contradiction_type (carried_forward_percentage_mismatch) and a lower confidence (medium vs. same-sentence count_percentage_mismatch's very_high), with evidence quoting the earlier sentence the denominator came from, so editors can tell a same-sentence match from a weaker cross-sentence inference. Known remaining gap, left deliberately unsolved per the audit's own conservatism: a bare percentage claim with no numerator at all ("the response rate was 45%") still can't be checked — there is nothing to divide, and guessing an implied count was explicitly out of scope. Verified by 5 new tests in tests/test_numerical_contradiction.py: true positive, two different-population false-positive guards, same-sentence non-regression, and most-recent-total-wins with a decoy total in between.</t>
         </is>
       </c>
     </row>
@@ -8833,9 +8843,9 @@
           <t>Documented before/after recall on a labeled sample for numerical contradictions; measured GPT-OSS call success rate under induced-failure testing; registry coverage matches ASCO's actual international submitter base.</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>In progress — 2026-08-19. OE-01 completed: shared sentence splitter (content_integrity.utils.split_sentences) now uses pysbd for abbreviation-aware segmentation, replacing the naive regex; verified against Fig./vs./e.g./i.v./no./decimal-adjacent cases in tests/test_utils.py, full suite green (268 passed) apart from the pre-existing, unrelated authorship-reporting failure. Remaining Phase 3 items not started: OE-09 (cross-sentence numeric linking), OE-07 (shared LLM client resilience), OE-08 (registry expansion).</t>
+      <c r="I6" s="0" t="inlineStr">
+        <is>
+          <t>Done — 2026-08-20. OE-01 completed 2026-08-19 (pysbd abbreviation-aware sentence splitter). OE-09: cross-sentence 'most recently stated N' carry-forward added to numerical_contradiction.py, conservatively gated against different-population false positives. OE-07: verified timeout/retry/backoff/shared-client/telemetry were already in place (from Phase 0) across all three GPT-OSS call sites; added the one genuine gap, content-addressed caching on IntelliHubGPTOSSClient, matching ClinicalTrialsGovClient's pattern. OE-08: registry coverage expanded to CTRI, DRKS, jRCT, IRCT, WHO ICTRP (format-validation only, no new live API clients); a real WHO-ICTRP-hyphen-eating bug was caught and fixed in the same pass. All three implemented in parallel by isolated subagents, independently audited (diff review + full-suite verification) and merged; 280 passed, 0 regressions, apart from the same one pre-existing, unrelated authorship-reporting failure carried since Phase 0. Separately discovered during this phase, not fixed: .gitignore's blanket *.xml rule also excludes several tests/fixtures/ files the suite depends on, so a fresh clone or git worktree gets 6 spurious test failures until those fixtures are copied in manually — a real repo-hygiene gap, flagged but left for a deliberate decision since *.xml is presumably also guarding against committing real (possibly sensitive) submission data.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update audit workbook for Phase 4: OE-04 partial, hidden fields surfaced
Records the corrected OE-04 diagnosis (targeted exact-hash-block fix,
not a full ANN/MinHash-LSH layer), the hidden-field surfacing work,
and the explicit product decision to redirect confidence calibration
to LLM-derived scoring instead of the blocked editor-history approach.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Content_Integrity_Pipeline_Audit.xlsx
+++ b/Content_Integrity_Pipeline_Audit.xlsx
@@ -7294,6 +7294,11 @@
       <c r="H6" s="10" t="inlineStr">
         <is>
           <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Partially resolved — 2026-08-20. Investigated before implementing: the approximate (shape/prefix) buckets and n-gram shingle index in template_matching_common.py were already capped and scale fine; the log's assumption that a whole new ANN/MinHash-LSH layer was needed did not hold up. The real uncapped gap was the exact-hash blocking layer across four call sites (template_matching_common.py, candidate_routes.py, title_templates.py, entity_normalized_template.py) - a single reused-boilerplate cluster (e.g. a repeated "trial in progress" abstract across years) produced a full O(k^2) clique with no cap; benchmarked at 12.5M pairs for 5,000 exact duplicates. Fixed with a shared _bounded_block_pairs() helper: unchanged full clique below the existing 50-member cap, a star off the smallest record id above it (O(k), verified sufficient for downstream union-find clustering connectivity). Classification logic untouched. Not a full ANN/MinHash-LSH layer as originally proposed - marked partial because multi-year cross-batch comparison itself is still not implemented (docs/prd.md still lists it as an open question), so this fix removes the compute-time cliff for whenever that comparison is turned on, but does not turn it on.</t>
         </is>
       </c>
     </row>
@@ -8890,6 +8895,11 @@
           <t>Template-detection runtime stays sub-quadratic-feeling as the corpus grows across years; editors report priority badges match their own sense of urgency; zero 'computed but hidden' fields remain undocumented.</t>
         </is>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>In progress — 2026-08-20. Two of three scope items done this pass, by isolated subagents in worktrees, independently reviewed (diff review + full-suite verification) and merged: OE-04 candidate-generation scaling (see Overengineering Log OE-04 for the corrected diagnosis - a smaller, more targeted fix than the log originally assumed); surfaced previously-computed-but-hidden fields (numerical calculated_value/difference/tolerance, clinical-trial registry_name/normalized_trial_id/format_valid/verification_status, and each detector's per-finding review_reason) into the JSON output via the existing Finding/_integrated_finding() plumbing - no workbook column added, since the Check Detail sheet deliberately excludes these three checks already (editors review them via content_integrity_results.json instead, per existing design). Third item, calibrating tortured-phrase confidence against real editor accept/reject history, was blocked (no such history exists in this repo) and redirected per explicit product decision: replaced the old fixed 0.98/0.87 heuristic split with a calibrated 0.0-1.0 confidence score from the existing GPT-OSS ContextValidator (only active when --validate-llm runs; falls back to the heuristic otherwise) rather than literal historical calibration. Full test suite green (284 passed) apart from the same one pre-existing, unrelated authorship-reporting failure carried since Phase 0. Editor-facing confidence-mapping calibration against real review history remains open and requires accumulated real editor decisions this project does not yet have.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="22"/>
     <row r="22" ht="15.75" customHeight="1" s="22"/>

</xml_diff>